<commit_message>
Add v4.1 PCB files and v3 3D prints
Add PCB package for QuantumDice_ESP32PCB v4.1 (BOM, CPL, Gerbers zip, PDF) and several Version 3 3D STL files (frame and display cups). Update 3D print and PCB README files with printing/assembly and PCB assembly notes (ESP32 processor, 6-layer, assemble both sides). Rename construction manual to "ConstructionManual [outdated].md", remove outdated PDF and IMU calibrator STL, and update Bill of Material Excel.
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/Quantum-Dice-by-UTwente/3D print files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/QD-prod/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D240F69-167D-0549-97BB-208FC9CADE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EB348C-ED9A-D94F-B158-C27E50C424D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11200" yWindow="600" windowWidth="34240" windowHeight="21140" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15960" activeTab="1" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="version2" sheetId="2" r:id="rId1"/>
+    <sheet name="version3.1" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -199,8 +200,126 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Aernout van Rossum</author>
+  </authors>
+  <commentList>
+    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{77A0812C-28AA-8449-8ACF-9FA47374E350}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">In rare situations the display module is Dead On Arrival (DOA). Order some extra display units
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0" shapeId="0" xr:uid="{54755A7F-74D4-144E-A19F-F99A712D832D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>3.7V lipo battery:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Size: maximum 50mm high/width. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">xx3048 -&gt; xx is thicknesss, 30 mm wide, 48 mm high
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Thickness: max 18 mm
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Capacitiy: &gt;1000 mAh. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Connector: JST-PH (2 pole), 2mm
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Check Polarity. See attached image
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="84">
   <si>
     <t>1.28 inch IPS Color TFT LCD Display Module 1.28" RGB LED Round Touch Screen GC9A01 Drive 4 Wire SPI Interface 240x240 PCB Board</t>
   </si>
@@ -401,6 +520,57 @@
   </si>
   <si>
     <t>https://github.com/qlab-utwente/Quantum-Dice-by-UTwente/tree/main/3D%20print%20files/Version%202</t>
+  </si>
+  <si>
+    <t>Quantum Dice display type 1</t>
+  </si>
+  <si>
+    <t>Cable set (see below for detailled specification)</t>
+  </si>
+  <si>
+    <t>ProcessorPCB ESP32 V4.0.1</t>
+  </si>
+  <si>
+    <t>https://nl.aliexpress.com/item/1005005998843790.html</t>
+  </si>
+  <si>
+    <t>USB-C cable with 6P connector (color B)</t>
+  </si>
+  <si>
+    <t>Optional NOT NEEDED when a complete set is ordered @Utwente</t>
+  </si>
+  <si>
+    <t>https://nederland.bossard.com/nl-nl/standaard-bevestigingsartikelen/schroeven/schroeven-met-interne-aandrijving/uls0000z0030006</t>
+  </si>
+  <si>
+    <t>https://nederland.bossard.com/nl-nl/standaard-bevestigingsartikelen/schroeven/schroeven-met-interne-aandrijving/798500k00030008</t>
+  </si>
+  <si>
+    <t>Polyamide 6.6 Pan head screws with Phillips cross recess (H), DIN 34812, M 3 X 8</t>
+  </si>
+  <si>
+    <t>buttonhead socket screws, M 3 X 6</t>
+  </si>
+  <si>
+    <t>order @ https://jlc3dp.com. Technique: Fused Deposition Modeling (FDM) material: TPU black</t>
+  </si>
+  <si>
+    <t>01A_Blck_TPU_V31_frame.stl</t>
+  </si>
+  <si>
+    <t>02A_Yellow_PLA_V31_display_cup_battery.stl</t>
+  </si>
+  <si>
+    <t>02B_Yellow_PLA_V31_display_cup_ESP32.stl</t>
+  </si>
+  <si>
+    <t>02C_Yellow_PLA_V31_display_cup_ESP32_cover.stl</t>
+  </si>
+  <si>
+    <t>02D_Blue_PLA_V31_display_cup_top_bottom.stl</t>
+  </si>
+  <si>
+    <t>02E_Red_PLA_V31_display_cup_left_right.stl</t>
   </si>
 </sst>
 </file>
@@ -501,7 +671,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -509,6 +679,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -570,6 +741,72 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>6400800</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Afbeelding 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F81B3F4C-E5C4-9F0B-64DA-B9A95040BFDD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="20334" t="67131"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13157200" y="1778000"/>
+          <a:ext cx="3632200" cy="1498600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1483,7 +1720,451 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C732FC4C-DAE6-4248-9E60-BA89F974A7C6}">
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="53.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="112.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="5"/>
+      <c r="E1" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10">
+        <f>$C$2*D10</f>
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11">
+        <f t="shared" ref="C11:C15" si="0">$C$2*D11</f>
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D14" s="4">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18">
+        <f t="shared" ref="C18:C19" si="1">$C$2*D18</f>
+        <v>12</v>
+      </c>
+      <c r="D18" s="4">
+        <v>6</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="1"/>
+        <v>48</v>
+      </c>
+      <c r="D19" s="4">
+        <f>4*6</f>
+        <v>24</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <f t="shared" ref="C22:C26" si="2">$C$2*D22</f>
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D26" s="4">
+        <v>1</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B28" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29">
+        <f>$C$2*D29</f>
+        <v>2</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30">
+        <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
+        <v>2</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="D31" s="4">
+        <v>4</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="D32" s="4">
+        <v>1</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="E33" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B38" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39">
+        <f t="shared" ref="C39:C42" si="4">$C$2*D39</f>
+        <v>55</v>
+      </c>
+      <c r="D39" s="4">
+        <f>55/2</f>
+        <v>27.5</v>
+      </c>
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="4"/>
+        <v>58</v>
+      </c>
+      <c r="D40" s="4">
+        <f>58/2</f>
+        <v>29</v>
+      </c>
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="4"/>
+        <v>66</v>
+      </c>
+      <c r="D41" s="4">
+        <v>33</v>
+      </c>
+      <c r="E41" s="6"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="4"/>
+        <v>126</v>
+      </c>
+      <c r="D42" s="4">
+        <f>126/2</f>
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E32" r:id="rId1" xr:uid="{888E8EFF-12A1-5647-A1DF-91A0B11A0742}"/>
+    <hyperlink ref="E31" r:id="rId2" xr:uid="{3E930678-8097-5743-A5D6-637CCB8D09F4}"/>
+    <hyperlink ref="E30" r:id="rId3" xr:uid="{B9BEE202-E8A4-2E4B-B3EA-F8F3B5495F4D}"/>
+    <hyperlink ref="E29" r:id="rId4" xr:uid="{ACB14C99-46CD-D843-B60D-4FDB2F746493}"/>
+    <hyperlink ref="E24" r:id="rId5" xr:uid="{847A1241-FDD5-2342-A0B6-623C025760E5}"/>
+    <hyperlink ref="E22" r:id="rId6" xr:uid="{58F8BEE9-79CA-D141-B04B-C80DEDF97435}"/>
+    <hyperlink ref="E33" r:id="rId7" xr:uid="{A4B5260C-1999-EE45-86CE-E77269A7D7C0}"/>
+    <hyperlink ref="E25" r:id="rId8" xr:uid="{36C7D458-A1BE-4E4C-973C-78793AF4FE94}"/>
+    <hyperlink ref="E26" r:id="rId9" xr:uid="{09394EB0-69D8-0143-9907-BFB2C5AF992C}"/>
+    <hyperlink ref="E23" r:id="rId10" xr:uid="{4BFEFEAC-F948-DB48-B0FD-182E9C3E2860}"/>
+    <hyperlink ref="E19" r:id="rId11" xr:uid="{49B33216-C293-6340-899F-341CD4072C86}"/>
+    <hyperlink ref="E18" r:id="rId12" xr:uid="{ECCD3433-8F01-F748-B2AA-FAC72BA0DF79}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId13"/>
+  <legacyDrawing r:id="rId14"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -1690,27 +2371,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
+    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1727,29 +2413,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
-    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Bill of Material quantum dice.xlsx
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/QD-prod/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EB348C-ED9A-D94F-B158-C27E50C424D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B605078E-10D8-A34C-B869-8181969C0C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15960" activeTab="1" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="1" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="version2" sheetId="2" r:id="rId1"/>
@@ -2156,15 +2156,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -2371,6 +2362,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
   <ds:schemaRefs>
@@ -2389,14 +2389,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2413,4 +2405,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Organize v4 files and docs
This change reorganizes the Version 4 print files into a dedicated Type A folder and archives older PCB design files for reference. It also updates the 3D print README to describe the Type A/Type B variants, adds display images, clarifies the variant differences, and fixes wording around support removal and BOM references. The BOM spreadsheet was refreshed and the Type B files are noted as still under construction.
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/QD-prod/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC63BA05-E2EA-4C4E-8B5A-82ACA00355B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C613AFB-801F-DF4F-9FE3-AA5C7E8B048A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="1" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="2" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="version2" sheetId="2" r:id="rId1"/>
-    <sheet name="version3.1" sheetId="4" r:id="rId2"/>
+    <sheet name="version 4.0-A" sheetId="4" r:id="rId2"/>
+    <sheet name="version 4.0-B" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -318,8 +319,126 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Aernout van Rossum</author>
+  </authors>
+  <commentList>
+    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{A9B79E6D-C9DB-9A47-910A-E2F29737A011}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">In rare situations the display module is Dead On Arrival (DOA). Order some extra display units
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0" shapeId="0" xr:uid="{62283A7F-8425-4144-8822-32526026DC64}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>3.7V lipo battery:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Size: maximum 50mm high/width. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">xx3048 -&gt; xx is thicknesss, 30 mm wide, 48 mm high
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Thickness: max 18 mm
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Capacitiy: &gt;1000 mAh. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Connector: JST-PH (2 pole), 2mm
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Check Polarity. See attached image
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="92">
   <si>
     <t>1.28 inch IPS Color TFT LCD Display Module 1.28" RGB LED Round Touch Screen GC9A01 Drive 4 Wire SPI Interface 240x240 PCB Board</t>
   </si>
@@ -519,9 +638,6 @@
     <t>For version 1.x.x the Blue top cup has an A and B indication</t>
   </si>
   <si>
-    <t>https://github.com/qlab-utwente/Quantum-Dice-by-UTwente/tree/main/3D%20print%20files/Version%202</t>
-  </si>
-  <si>
     <t>Quantum Dice display type 1</t>
   </si>
   <si>
@@ -546,25 +662,58 @@
     <t>buttonhead socket screws, M 3 X 6</t>
   </si>
   <si>
-    <t>order @ https://jlc3dp.com. Technique: Fused Deposition Modeling (FDM) material: TPU black</t>
-  </si>
-  <si>
-    <t>01A_Blck_TPU_V31_frame.stl</t>
-  </si>
-  <si>
-    <t>02A_Yellow_PLA_V31_display_cup_battery.stl</t>
-  </si>
-  <si>
-    <t>02B_Yellow_PLA_V31_display_cup_ESP32.stl</t>
-  </si>
-  <si>
-    <t>02C_Yellow_PLA_V31_display_cup_ESP32_cover.stl</t>
-  </si>
-  <si>
-    <t>02D_Blue_PLA_V31_display_cup_top_bottom.stl</t>
-  </si>
-  <si>
-    <t>02E_Red_PLA_V31_display_cup_left_right.stl</t>
+    <t>02A_Yellow_PLA_V40-A_display_cup_battery.stl</t>
+  </si>
+  <si>
+    <t>02B_Yellow_PLA_V40-A_display_cup_ESP32.stl</t>
+  </si>
+  <si>
+    <t>02C_Yellow_PLA_V40-A_display_cup_ESP32_cover.stl</t>
+  </si>
+  <si>
+    <t>02D_Blue_PLA_V40-A_display_cup_top_bottom.stl</t>
+  </si>
+  <si>
+    <t>02E_Red_PLA_V40-A_display_cup_left_right.stl</t>
+  </si>
+  <si>
+    <t>01A_Blck_TPU_V40_frame.stl</t>
+  </si>
+  <si>
+    <t>Cable set, containing:</t>
+  </si>
+  <si>
+    <t>Support material</t>
+  </si>
+  <si>
+    <t>02A_Yellow_PLA_V40-B_display_cup_battery.stl</t>
+  </si>
+  <si>
+    <t>02B_Yellow_PLA_V40-B_display_cup_ESP32.stl</t>
+  </si>
+  <si>
+    <t>02C_Yellow_PLA_V40-B_display_cup_ESP32_cover.stl</t>
+  </si>
+  <si>
+    <t>02D_Blue_PLA_V40-B_display_cup_top_bottom.stl</t>
+  </si>
+  <si>
+    <t>02E_Red_PLA_V40-B_display_cup_left_right.stl</t>
+  </si>
+  <si>
+    <t>https://nl.aliexpress.com/item/1005010527932589.html</t>
+  </si>
+  <si>
+    <t>See 3D print folder</t>
+  </si>
+  <si>
+    <t>See 3D print folder. Order @ https://jlc3dp.com. Technique: Fused Deposition Modeling (FDM) material: TPU black</t>
+  </si>
+  <si>
+    <t>pan head, M1.7, 4mm</t>
+  </si>
+  <si>
+    <t>https://nl.aliexpress.com/item/33043885403.html</t>
   </si>
 </sst>
 </file>
@@ -574,7 +723,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;€&quot;\ * #,##0.00_);_(&quot;€&quot;\ * \(#,##0.00\);_(&quot;€&quot;\ * &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -642,6 +791,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -665,7 +820,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -674,6 +829,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -763,6 +919,72 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F81B3F4C-E5C4-9F0B-64DA-B9A95040BFDD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="20334" t="67131"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13195300" y="1282700"/>
+          <a:ext cx="3632200" cy="1498600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>6438900</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>673100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Afbeelding 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68646307-5D43-7641-8849-EED703A9644F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1196,8 +1418,8 @@
       <c r="D10" s="4">
         <v>1</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>66</v>
+      <c r="E10" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -1211,8 +1433,8 @@
       <c r="D11" s="4">
         <v>1</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>66</v>
+      <c r="E11" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1226,8 +1448,8 @@
       <c r="D12" s="4">
         <v>2</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>66</v>
+      <c r="E12" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1241,8 +1463,8 @@
       <c r="D13" s="4">
         <v>1</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>66</v>
+      <c r="E13" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1256,8 +1478,8 @@
       <c r="D14" s="4">
         <v>1</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>66</v>
+      <c r="E14" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1271,8 +1493,8 @@
       <c r="D15" s="4">
         <v>2</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>66</v>
+      <c r="E15" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1286,8 +1508,8 @@
       <c r="D16" s="4">
         <v>2</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>66</v>
+      <c r="E16" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
@@ -1301,8 +1523,8 @@
       <c r="D17" s="4">
         <v>4</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>66</v>
+      <c r="E17" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
@@ -1316,8 +1538,8 @@
       <c r="D18" s="4">
         <v>1</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>66</v>
+      <c r="E18" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
@@ -1331,8 +1553,8 @@
       <c r="D19" s="4">
         <v>1</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>66</v>
+      <c r="E19" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
@@ -1743,7 +1965,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1770,7 +1992,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C10">
         <f>$C$2*D10</f>
@@ -1780,12 +2002,12 @@
         <v>1</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C11">
         <f t="shared" ref="C11:C15" si="0">$C$2*D11</f>
@@ -1794,11 +2016,13 @@
       <c r="D11" s="4">
         <v>1</v>
       </c>
-      <c r="E11" s="1"/>
+      <c r="E11" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C12">
         <f t="shared" si="0"/>
@@ -1807,11 +2031,13 @@
       <c r="D12" s="4">
         <v>1</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
@@ -1820,11 +2046,13 @@
       <c r="D13" s="4">
         <v>1</v>
       </c>
-      <c r="E13" s="1"/>
+      <c r="E13" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
@@ -1833,11 +2061,13 @@
       <c r="D14" s="4">
         <v>2</v>
       </c>
-      <c r="E14" s="1"/>
+      <c r="E14" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -1846,7 +2076,9 @@
       <c r="D15" s="4">
         <v>2</v>
       </c>
-      <c r="E15" s="1"/>
+      <c r="E15" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" s="2" t="s">
@@ -1870,7 +2102,7 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19">
         <f t="shared" si="1"/>
@@ -1881,7 +2113,7 @@
         <v>24</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
@@ -1906,7 +2138,7 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C23">
         <f t="shared" si="2"/>
@@ -1921,7 +2153,7 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C24">
         <f t="shared" si="2"/>
@@ -1951,7 +2183,7 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C26">
         <f t="shared" si="2"/>
@@ -1961,15 +2193,15 @@
         <v>1</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="E28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
@@ -2039,7 +2271,7 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" s="2" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -2138,18 +2370,440 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BC8621-1476-984A-8C7C-E2A66EAE4988}">
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="53.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="112.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="5"/>
+      <c r="E1" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10">
+        <f>$C$2*D10</f>
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11">
+        <f t="shared" ref="C11:C15" si="0">$C$2*D11</f>
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D14" s="4">
+        <v>2</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18">
+        <f t="shared" ref="C18:C19" si="1">$C$2*D18</f>
+        <v>12</v>
+      </c>
+      <c r="D18" s="4">
+        <v>6</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="1"/>
+        <v>48</v>
+      </c>
+      <c r="D19" s="4">
+        <f>4*6</f>
+        <v>24</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <f t="shared" ref="C22:C26" si="2">$C$2*D22</f>
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D26" s="4">
+        <v>1</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29">
+        <f>$C$2*D29</f>
+        <v>2</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30">
+        <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
+        <v>2</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="D31" s="4">
+        <v>4</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="D32" s="4">
+        <v>1</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="E33" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B38" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39">
+        <f t="shared" ref="C39:C42" si="4">$C$2*D39</f>
+        <v>55</v>
+      </c>
+      <c r="D39" s="4">
+        <f>55/2</f>
+        <v>27.5</v>
+      </c>
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="4"/>
+        <v>58</v>
+      </c>
+      <c r="D40" s="4">
+        <f>58/2</f>
+        <v>29</v>
+      </c>
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="4"/>
+        <v>66</v>
+      </c>
+      <c r="D41" s="4">
+        <v>33</v>
+      </c>
+      <c r="E41" s="6"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="4"/>
+        <v>126</v>
+      </c>
+      <c r="D42" s="4">
+        <f>126/2</f>
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E32" r:id="rId1" xr:uid="{43B90185-49CE-6844-B356-30E2993200E7}"/>
+    <hyperlink ref="E31" r:id="rId2" xr:uid="{DACA1E50-ACCF-2C47-B3F6-63D781231215}"/>
+    <hyperlink ref="E30" r:id="rId3" xr:uid="{E018907D-0983-DA49-9C2A-A6966B678DD1}"/>
+    <hyperlink ref="E29" r:id="rId4" xr:uid="{ECE159F7-FA27-204B-ADCB-D72AF272AAED}"/>
+    <hyperlink ref="E24" r:id="rId5" xr:uid="{21D1320F-2848-034D-A80B-78ABF00DB9F7}"/>
+    <hyperlink ref="E33" r:id="rId6" xr:uid="{377FC54D-F5F7-BB42-9648-0E1D832CFB0F}"/>
+    <hyperlink ref="E25" r:id="rId7" xr:uid="{A8433DAF-09BF-3D4B-A2FA-7BBB9ABDA4AC}"/>
+    <hyperlink ref="E26" r:id="rId8" xr:uid="{D0F972C1-8472-4E4B-A8C6-89C6B77629C8}"/>
+    <hyperlink ref="E23" r:id="rId9" xr:uid="{F304845B-F5B1-584B-A378-23BE1667DECC}"/>
+    <hyperlink ref="E18" r:id="rId10" xr:uid="{30CCA9EB-3FF1-B949-9D54-13A168189E0E}"/>
+    <hyperlink ref="E22" r:id="rId11" xr:uid="{B10439B4-1A44-2848-A60E-C4412FAE6F19}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId12"/>
+  <legacyDrawing r:id="rId13"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -2356,7 +3010,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2365,24 +3019,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
-    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2401,10 +3049,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
+    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update assembly docs and images
Refresh the Quantum Dice construction guide with cleaner markdown formatting, add the cable image to the assembly section, rename the battery image to match the project conventions, and fix the README link to the construction manual.
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/QD-prod/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C613AFB-801F-DF4F-9FE3-AA5C7E8B048A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A4EFE3-2E6E-6547-B276-EBBC9242E528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="2" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="97">
   <si>
     <t>1.28 inch IPS Color TFT LCD Display Module 1.28" RGB LED Round Touch Screen GC9A01 Drive 4 Wire SPI Interface 240x240 PCB Board</t>
   </si>
@@ -714,6 +714,21 @@
   </si>
   <si>
     <t>https://nl.aliexpress.com/item/33043885403.html</t>
+  </si>
+  <si>
+    <t>DESIGN DISPALAY CUPS V4.0-B are not finished yet!</t>
+  </si>
+  <si>
+    <t>https://nl.aliexpress.com/item/1005007271132722.html</t>
+  </si>
+  <si>
+    <t>8Pin 60mm AWM 20624 80°C 60V VW-1 0,5mm FFC Flexible Flat Cable (Forward)</t>
+  </si>
+  <si>
+    <t>8Pin 100mm AWM 20624 80°C 60V VW-1 0,5mm FFC Flexible Flat Cable (Forward</t>
+  </si>
+  <si>
+    <t>8Pin 150mm AWM 20624 80°C 60V VW-1 0,5mm FFC Flexible Flat Cable (Forward)</t>
   </si>
 </sst>
 </file>
@@ -798,12 +813,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -820,7 +841,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -830,6 +851,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2221,7 +2243,7 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
@@ -2231,12 +2253,12 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="C31">
         <f t="shared" si="3"/>
@@ -2246,12 +2268,12 @@
         <v>4</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>24</v>
+        <v>96</v>
       </c>
       <c r="C32">
         <f t="shared" si="3"/>
@@ -2261,13 +2283,11 @@
         <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>5</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="E33" s="1" t="s">
-        <v>63</v>
-      </c>
+      <c r="E33" s="1"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" s="2" t="s">
@@ -2351,22 +2371,18 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E32" r:id="rId1" xr:uid="{888E8EFF-12A1-5647-A1DF-91A0B11A0742}"/>
-    <hyperlink ref="E31" r:id="rId2" xr:uid="{3E930678-8097-5743-A5D6-637CCB8D09F4}"/>
-    <hyperlink ref="E30" r:id="rId3" xr:uid="{B9BEE202-E8A4-2E4B-B3EA-F8F3B5495F4D}"/>
-    <hyperlink ref="E29" r:id="rId4" xr:uid="{ACB14C99-46CD-D843-B60D-4FDB2F746493}"/>
-    <hyperlink ref="E24" r:id="rId5" xr:uid="{847A1241-FDD5-2342-A0B6-623C025760E5}"/>
-    <hyperlink ref="E22" r:id="rId6" xr:uid="{58F8BEE9-79CA-D141-B04B-C80DEDF97435}"/>
-    <hyperlink ref="E33" r:id="rId7" xr:uid="{A4B5260C-1999-EE45-86CE-E77269A7D7C0}"/>
-    <hyperlink ref="E25" r:id="rId8" xr:uid="{36C7D458-A1BE-4E4C-973C-78793AF4FE94}"/>
-    <hyperlink ref="E26" r:id="rId9" xr:uid="{09394EB0-69D8-0143-9907-BFB2C5AF992C}"/>
-    <hyperlink ref="E23" r:id="rId10" xr:uid="{4BFEFEAC-F948-DB48-B0FD-182E9C3E2860}"/>
-    <hyperlink ref="E19" r:id="rId11" xr:uid="{49B33216-C293-6340-899F-341CD4072C86}"/>
-    <hyperlink ref="E18" r:id="rId12" xr:uid="{8A21DB98-CC3E-B244-A5CF-BA35B77F2405}"/>
+    <hyperlink ref="E29" r:id="rId1" xr:uid="{ACB14C99-46CD-D843-B60D-4FDB2F746493}"/>
+    <hyperlink ref="E24" r:id="rId2" xr:uid="{847A1241-FDD5-2342-A0B6-623C025760E5}"/>
+    <hyperlink ref="E22" r:id="rId3" xr:uid="{58F8BEE9-79CA-D141-B04B-C80DEDF97435}"/>
+    <hyperlink ref="E25" r:id="rId4" xr:uid="{36C7D458-A1BE-4E4C-973C-78793AF4FE94}"/>
+    <hyperlink ref="E26" r:id="rId5" xr:uid="{09394EB0-69D8-0143-9907-BFB2C5AF992C}"/>
+    <hyperlink ref="E23" r:id="rId6" xr:uid="{4BFEFEAC-F948-DB48-B0FD-182E9C3E2860}"/>
+    <hyperlink ref="E19" r:id="rId7" xr:uid="{49B33216-C293-6340-899F-341CD4072C86}"/>
+    <hyperlink ref="E18" r:id="rId8" xr:uid="{8A21DB98-CC3E-B244-A5CF-BA35B77F2405}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId13"/>
-  <legacyDrawing r:id="rId14"/>
+  <drawing r:id="rId9"/>
+  <legacyDrawing r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -2404,6 +2420,9 @@
       <c r="C2">
         <v>2</v>
       </c>
+      <c r="E2" s="9" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
@@ -2655,7 +2674,7 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
@@ -2665,12 +2684,12 @@
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="C31">
         <f t="shared" si="3"/>
@@ -2680,12 +2699,12 @@
         <v>4</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>24</v>
+        <v>96</v>
       </c>
       <c r="C32">
         <f t="shared" si="3"/>
@@ -2695,13 +2714,11 @@
         <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>5</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="E33" s="1" t="s">
-        <v>63</v>
-      </c>
+      <c r="E33" s="1"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" s="2" t="s">
@@ -2785,25 +2802,41 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E32" r:id="rId1" xr:uid="{43B90185-49CE-6844-B356-30E2993200E7}"/>
-    <hyperlink ref="E31" r:id="rId2" xr:uid="{DACA1E50-ACCF-2C47-B3F6-63D781231215}"/>
-    <hyperlink ref="E30" r:id="rId3" xr:uid="{E018907D-0983-DA49-9C2A-A6966B678DD1}"/>
-    <hyperlink ref="E29" r:id="rId4" xr:uid="{ECE159F7-FA27-204B-ADCB-D72AF272AAED}"/>
-    <hyperlink ref="E24" r:id="rId5" xr:uid="{21D1320F-2848-034D-A80B-78ABF00DB9F7}"/>
-    <hyperlink ref="E33" r:id="rId6" xr:uid="{377FC54D-F5F7-BB42-9648-0E1D832CFB0F}"/>
-    <hyperlink ref="E25" r:id="rId7" xr:uid="{A8433DAF-09BF-3D4B-A2FA-7BBB9ABDA4AC}"/>
-    <hyperlink ref="E26" r:id="rId8" xr:uid="{D0F972C1-8472-4E4B-A8C6-89C6B77629C8}"/>
-    <hyperlink ref="E23" r:id="rId9" xr:uid="{F304845B-F5B1-584B-A378-23BE1667DECC}"/>
-    <hyperlink ref="E18" r:id="rId10" xr:uid="{30CCA9EB-3FF1-B949-9D54-13A168189E0E}"/>
-    <hyperlink ref="E22" r:id="rId11" xr:uid="{B10439B4-1A44-2848-A60E-C4412FAE6F19}"/>
+    <hyperlink ref="E24" r:id="rId1" xr:uid="{21D1320F-2848-034D-A80B-78ABF00DB9F7}"/>
+    <hyperlink ref="E25" r:id="rId2" xr:uid="{A8433DAF-09BF-3D4B-A2FA-7BBB9ABDA4AC}"/>
+    <hyperlink ref="E26" r:id="rId3" xr:uid="{D0F972C1-8472-4E4B-A8C6-89C6B77629C8}"/>
+    <hyperlink ref="E23" r:id="rId4" xr:uid="{F304845B-F5B1-584B-A378-23BE1667DECC}"/>
+    <hyperlink ref="E18" r:id="rId5" xr:uid="{30CCA9EB-3FF1-B949-9D54-13A168189E0E}"/>
+    <hyperlink ref="E22" r:id="rId6" xr:uid="{B10439B4-1A44-2848-A60E-C4412FAE6F19}"/>
+    <hyperlink ref="E29" r:id="rId7" xr:uid="{0A19CB42-3C63-F240-B3E6-8E0737F8F871}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId12"/>
-  <legacyDrawing r:id="rId13"/>
+  <drawing r:id="rId8"/>
+  <legacyDrawing r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -3010,27 +3043,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
+    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3047,29 +3085,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
-    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add V4 Type A STL files and update BOM
Add three 3D-print STL files for Version 4 Type A: 02D_Yellow_PLA_V40-A_battery_holder.stl, FPC tooltje ESP32.stl, and FPC tooltje display.stl. Update the Bill of Material spreadsheet (Bill of Material quantum dice.xlsx) to reflect these additions.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/QD-prod/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D762E6-ED40-7341-92AB-E7520C344FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A65745-7B50-7D4B-A2B7-C0C04C2AA397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="1" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" activeTab="2" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="version2" sheetId="2" r:id="rId1"/>
@@ -207,7 +207,7 @@
     <author>Aernout van Rossum</author>
   </authors>
   <commentList>
-    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{77A0812C-28AA-8449-8ACF-9FA47374E350}">
+    <comment ref="B26" authorId="0" shapeId="0" xr:uid="{77A0812C-28AA-8449-8ACF-9FA47374E350}">
       <text>
         <r>
           <rPr>
@@ -221,7 +221,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B25" authorId="0" shapeId="0" xr:uid="{54755A7F-74D4-144E-A19F-F99A712D832D}">
+    <comment ref="B29" authorId="0" shapeId="0" xr:uid="{54755A7F-74D4-144E-A19F-F99A712D832D}">
       <text>
         <r>
           <rPr>
@@ -325,7 +325,7 @@
     <author>Aernout van Rossum</author>
   </authors>
   <commentList>
-    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{A9B79E6D-C9DB-9A47-910A-E2F29737A011}">
+    <comment ref="B26" authorId="0" shapeId="0" xr:uid="{A9B79E6D-C9DB-9A47-910A-E2F29737A011}">
       <text>
         <r>
           <rPr>
@@ -339,7 +339,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B25" authorId="0" shapeId="0" xr:uid="{62283A7F-8425-4144-8822-32526026DC64}">
+    <comment ref="B29" authorId="0" shapeId="0" xr:uid="{62283A7F-8425-4144-8822-32526026DC64}">
       <text>
         <r>
           <rPr>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="108">
   <si>
     <t>1.28 inch IPS Color TFT LCD Display Module 1.28" RGB LED Round Touch Screen GC9A01 Drive 4 Wire SPI Interface 240x240 PCB Board</t>
   </si>
@@ -744,6 +744,24 @@
   </si>
   <si>
     <t>TPU  incl TPU support everywhere</t>
+  </si>
+  <si>
+    <t>02D_Yellow_PLA_V40-A_battery_holder.stl</t>
+  </si>
+  <si>
+    <t>FPC tooltje display.stl</t>
+  </si>
+  <si>
+    <t>FPC tooltje ESP32.stl</t>
+  </si>
+  <si>
+    <t>See 3D print folder; device to insert FPC cables to ESP32 board</t>
+  </si>
+  <si>
+    <t>See 3D print folder; device to insert FPC cables to displays</t>
+  </si>
+  <si>
+    <t>Optional</t>
   </si>
 </sst>
 </file>
@@ -1975,7 +1993,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C732FC4C-DAE6-4248-9E60-BA89F974A7C6}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -2047,7 +2065,7 @@
         <v>74</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:C15" si="0">$C$2*D11</f>
+        <f t="shared" ref="C11:C16" si="0">$C$2*D11</f>
         <v>2</v>
       </c>
       <c r="D11" s="4">
@@ -2089,14 +2107,14 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>88</v>
@@ -2104,7 +2122,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -2117,283 +2135,323 @@
         <v>88</v>
       </c>
     </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18">
-        <f t="shared" ref="C18:C19" si="1">$C$2*D18</f>
-        <v>12</v>
-      </c>
-      <c r="D18" s="4">
-        <v>6</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>18</v>
+        <v>103</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22">
+        <f t="shared" ref="C22:C23" si="1">$C$2*D22</f>
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
         <v>73</v>
       </c>
-      <c r="C19">
+      <c r="C23">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D23" s="4">
         <f>4*6</f>
         <v>24</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21" s="2" t="s">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <f t="shared" ref="C22:C26" si="2">$C$2*D22</f>
-        <v>12</v>
-      </c>
-      <c r="D22" s="4">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D24" s="4">
-        <v>1</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D25" s="4">
-        <v>1</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C26">
+        <f t="shared" ref="C26:C30" si="2">$C$2*D26</f>
+        <v>12</v>
+      </c>
+      <c r="D26" s="4">
+        <v>6</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="D26" s="4">
-        <v>1</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>69</v>
+      <c r="D27" s="4">
+        <v>1</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B28" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E28" t="s">
-        <v>71</v>
+      <c r="B28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D28" s="4">
+        <v>1</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C29">
-        <f>$C$2*D29</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33">
+        <f>$C$2*D33</f>
+        <v>2</v>
+      </c>
+      <c r="D33" s="4">
+        <v>1</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
         <v>94</v>
       </c>
-      <c r="C30">
-        <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
-        <v>2</v>
-      </c>
-      <c r="D30" s="4">
-        <v>1</v>
-      </c>
-      <c r="E30" s="1" t="s">
+      <c r="C34">
+        <f t="shared" ref="C34:C36" si="3">$C$2*D34</f>
+        <v>2</v>
+      </c>
+      <c r="D34" s="4">
+        <v>1</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B31" t="s">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
         <v>95</v>
       </c>
-      <c r="C31">
+      <c r="C35">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D35" s="4">
         <v>4</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B32" t="s">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
         <v>96</v>
       </c>
-      <c r="C32">
+      <c r="C36">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="D32" s="4">
-        <v>1</v>
-      </c>
-      <c r="E32" s="1" t="s">
+      <c r="D36" s="4">
+        <v>1</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B36" s="3" t="s">
-        <v>2</v>
-      </c>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="E37" s="1"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B39" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B39" t="s">
+    <row r="43" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
         <v>98</v>
       </c>
-      <c r="C39">
-        <f t="shared" ref="C39:C42" si="4">$C$2*D39</f>
+      <c r="C43">
+        <f t="shared" ref="C43:C46" si="4">$C$2*D43</f>
         <v>48</v>
       </c>
-      <c r="D39" s="4">
+      <c r="D43" s="4">
         <f>48/2</f>
         <v>24</v>
       </c>
-      <c r="E39" s="6"/>
-    </row>
-    <row r="40" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B40" t="s">
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
         <v>99</v>
       </c>
-      <c r="C40">
+      <c r="C44">
         <f t="shared" si="4"/>
         <v>48</v>
       </c>
-      <c r="D40" s="4">
+      <c r="D44" s="4">
         <f>48/2</f>
         <v>24</v>
       </c>
-      <c r="E40" s="6"/>
-    </row>
-    <row r="41" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B41" t="s">
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
         <v>100</v>
       </c>
-      <c r="C41">
+      <c r="C45">
         <f t="shared" si="4"/>
-        <v>59</v>
-      </c>
-      <c r="D41" s="4">
-        <f>59/2</f>
-        <v>29.5</v>
-      </c>
-      <c r="E41" s="6"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B42" t="s">
+        <v>72</v>
+      </c>
+      <c r="D45" s="4">
+        <f>72/2</f>
+        <v>36</v>
+      </c>
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
         <v>101</v>
       </c>
-      <c r="C42">
+      <c r="C46">
         <f t="shared" si="4"/>
         <v>166</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D46" s="4">
         <f>166/2</f>
         <v>83</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E24" r:id="rId1" xr:uid="{847A1241-FDD5-2342-A0B6-623C025760E5}"/>
-    <hyperlink ref="E22" r:id="rId2" xr:uid="{58F8BEE9-79CA-D141-B04B-C80DEDF97435}"/>
-    <hyperlink ref="E25" r:id="rId3" xr:uid="{36C7D458-A1BE-4E4C-973C-78793AF4FE94}"/>
-    <hyperlink ref="E26" r:id="rId4" xr:uid="{09394EB0-69D8-0143-9907-BFB2C5AF992C}"/>
-    <hyperlink ref="E23" r:id="rId5" xr:uid="{4BFEFEAC-F948-DB48-B0FD-182E9C3E2860}"/>
-    <hyperlink ref="E19" r:id="rId6" xr:uid="{49B33216-C293-6340-899F-341CD4072C86}"/>
-    <hyperlink ref="E18" r:id="rId7" xr:uid="{8A21DB98-CC3E-B244-A5CF-BA35B77F2405}"/>
+    <hyperlink ref="E28" r:id="rId1" xr:uid="{847A1241-FDD5-2342-A0B6-623C025760E5}"/>
+    <hyperlink ref="E26" r:id="rId2" xr:uid="{58F8BEE9-79CA-D141-B04B-C80DEDF97435}"/>
+    <hyperlink ref="E29" r:id="rId3" xr:uid="{36C7D458-A1BE-4E4C-973C-78793AF4FE94}"/>
+    <hyperlink ref="E30" r:id="rId4" xr:uid="{09394EB0-69D8-0143-9907-BFB2C5AF992C}"/>
+    <hyperlink ref="E27" r:id="rId5" xr:uid="{4BFEFEAC-F948-DB48-B0FD-182E9C3E2860}"/>
+    <hyperlink ref="E23" r:id="rId6" xr:uid="{49B33216-C293-6340-899F-341CD4072C86}"/>
+    <hyperlink ref="E22" r:id="rId7" xr:uid="{8A21DB98-CC3E-B244-A5CF-BA35B77F2405}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId8"/>
@@ -2403,7 +2461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BC8621-1476-984A-8C7C-E2A66EAE4988}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -2478,7 +2536,7 @@
         <v>82</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:C15" si="0">$C$2*D11</f>
+        <f t="shared" ref="C11:C16" si="0">$C$2*D11</f>
         <v>2</v>
       </c>
       <c r="D11" s="4">
@@ -2520,14 +2578,14 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>88</v>
@@ -2535,7 +2593,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -2548,281 +2606,322 @@
         <v>88</v>
       </c>
     </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18">
-        <f t="shared" ref="C18:C19" si="1">$C$2*D18</f>
-        <v>12</v>
-      </c>
-      <c r="D18" s="4">
-        <v>6</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>18</v>
+        <v>103</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22">
+        <f t="shared" ref="C22:C23" si="1">$C$2*D22</f>
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
         <v>90</v>
       </c>
-      <c r="C19">
+      <c r="C23">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D23" s="4">
         <f>4*6</f>
         <v>24</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21" s="2" t="s">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <f t="shared" ref="C22:C26" si="2">$C$2*D22</f>
-        <v>12</v>
-      </c>
-      <c r="D22" s="4">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D24" s="4">
-        <v>1</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25">
-        <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="D25" s="4">
-        <v>1</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C26">
+        <f t="shared" ref="C26:C30" si="2">$C$2*D26</f>
+        <v>12</v>
+      </c>
+      <c r="D26" s="4">
+        <v>6</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="D26" s="4">
-        <v>1</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>69</v>
+      <c r="D27" s="4">
+        <v>1</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B28" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E28" t="s">
-        <v>71</v>
+      <c r="B28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D28" s="4">
+        <v>1</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C29">
-        <f>$C$2*D29</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33">
+        <f>$C$2*D33</f>
+        <v>2</v>
+      </c>
+      <c r="D33" s="4">
+        <v>1</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
         <v>94</v>
       </c>
-      <c r="C30">
-        <f t="shared" ref="C30:C32" si="3">$C$2*D30</f>
-        <v>2</v>
-      </c>
-      <c r="D30" s="4">
-        <v>1</v>
-      </c>
-      <c r="E30" s="1" t="s">
+      <c r="C34">
+        <f t="shared" ref="C34:C36" si="3">$C$2*D34</f>
+        <v>2</v>
+      </c>
+      <c r="D34" s="4">
+        <v>1</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B31" t="s">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
         <v>95</v>
       </c>
-      <c r="C31">
+      <c r="C35">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D35" s="4">
         <v>4</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B32" t="s">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
         <v>96</v>
       </c>
-      <c r="C32">
+      <c r="C36">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="D32" s="4">
-        <v>1</v>
-      </c>
-      <c r="E32" s="1" t="s">
+      <c r="D36" s="4">
+        <v>1</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B36" s="3" t="s">
-        <v>2</v>
-      </c>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="E37" s="1"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B39" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B39" t="s">
+    <row r="43" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
         <v>48</v>
       </c>
-      <c r="C39">
-        <f t="shared" ref="C39:C42" si="4">$C$2*D39</f>
-        <v>55</v>
-      </c>
-      <c r="D39" s="4">
-        <f>55/2</f>
-        <v>27.5</v>
-      </c>
-      <c r="E39" s="6"/>
-    </row>
-    <row r="40" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B40" t="s">
+      <c r="C43">
+        <f t="shared" ref="C43:C46" si="4">$C$2*D43</f>
+        <v>48</v>
+      </c>
+      <c r="D43" s="4">
+        <f>48/2</f>
+        <v>24</v>
+      </c>
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
         <v>49</v>
       </c>
-      <c r="C40">
+      <c r="C44">
         <f t="shared" si="4"/>
-        <v>58</v>
-      </c>
-      <c r="D40" s="4">
-        <f>58/2</f>
-        <v>29</v>
-      </c>
-      <c r="E40" s="6"/>
-    </row>
-    <row r="41" spans="2:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B41" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44" s="4">
+        <f>48/2</f>
+        <v>24</v>
+      </c>
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
         <v>50</v>
       </c>
-      <c r="C41">
+      <c r="C45">
         <f t="shared" si="4"/>
-        <v>66</v>
-      </c>
-      <c r="D41" s="4">
-        <v>33</v>
-      </c>
-      <c r="E41" s="6"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B42" t="s">
+        <v>72</v>
+      </c>
+      <c r="D45" s="4">
+        <f>72/2</f>
+        <v>36</v>
+      </c>
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
         <v>51</v>
       </c>
-      <c r="C42">
+      <c r="C46">
         <f t="shared" si="4"/>
-        <v>126</v>
-      </c>
-      <c r="D42" s="4">
-        <f>126/2</f>
-        <v>63</v>
+        <v>166</v>
+      </c>
+      <c r="D46" s="4">
+        <f>166/2</f>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E24" r:id="rId1" xr:uid="{21D1320F-2848-034D-A80B-78ABF00DB9F7}"/>
-    <hyperlink ref="E25" r:id="rId2" xr:uid="{A8433DAF-09BF-3D4B-A2FA-7BBB9ABDA4AC}"/>
-    <hyperlink ref="E26" r:id="rId3" xr:uid="{D0F972C1-8472-4E4B-A8C6-89C6B77629C8}"/>
-    <hyperlink ref="E23" r:id="rId4" xr:uid="{F304845B-F5B1-584B-A378-23BE1667DECC}"/>
-    <hyperlink ref="E18" r:id="rId5" xr:uid="{30CCA9EB-3FF1-B949-9D54-13A168189E0E}"/>
-    <hyperlink ref="E22" r:id="rId6" xr:uid="{B10439B4-1A44-2848-A60E-C4412FAE6F19}"/>
+    <hyperlink ref="E28" r:id="rId1" xr:uid="{21D1320F-2848-034D-A80B-78ABF00DB9F7}"/>
+    <hyperlink ref="E29" r:id="rId2" xr:uid="{A8433DAF-09BF-3D4B-A2FA-7BBB9ABDA4AC}"/>
+    <hyperlink ref="E30" r:id="rId3" xr:uid="{D0F972C1-8472-4E4B-A8C6-89C6B77629C8}"/>
+    <hyperlink ref="E27" r:id="rId4" xr:uid="{F304845B-F5B1-584B-A378-23BE1667DECC}"/>
+    <hyperlink ref="E22" r:id="rId5" xr:uid="{30CCA9EB-3FF1-B949-9D54-13A168189E0E}"/>
+    <hyperlink ref="E26" r:id="rId6" xr:uid="{B10439B4-1A44-2848-A60E-C4412FAE6F19}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId7"/>
@@ -2831,6 +2930,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -3037,27 +3156,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
+    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3074,29 +3198,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
-    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>